<commit_message>
feat: plantilla Excel soporta gastos e ingresos en una sola carga
- Nueva columna Tipo (Gasto/Ingreso) con validación dropdown
- Handler detecta automáticamente formato 6 o 7 columnas (retrocompatible)
- Resumen de carga muestra gastos e ingresos por separado
- Plantilla regenerada con ejemplo de ingreso

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantilla_gastos.xlsx
+++ b/public/plantilla_gastos.xlsx
@@ -4,16 +4,16 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Gastos" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Movimientos" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
-  <si>
-    <t>PLANTILLA NETO — Carga de Gastos Históricos. Completa cada fila con un gasto. Las columnas Categoría, Método de Pago y Banco son opcionales (NETO las asigna automáticamente con IA).</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
+  <si>
+    <t>PLANTILLA NETO — Carga de Gastos e Ingresos Históricos. Completa cada fila con un movimiento. Las columnas Tipo, Categoría, Método de Pago y Banco son opcionales (NETO las asigna automáticamente con IA).</t>
   </si>
   <si>
     <t>Fecha</t>
@@ -25,6 +25,9 @@
     <t>Comercio / Descripción</t>
   </si>
   <si>
+    <t>Tipo</t>
+  </si>
+  <si>
     <t>Categoría</t>
   </si>
   <si>
@@ -40,6 +43,9 @@
     <t>Supermercado Metro</t>
   </si>
   <si>
+    <t>Gasto</t>
+  </si>
+  <si>
     <t>Alimentación</t>
   </si>
   <si>
@@ -59,6 +65,21 @@
   </si>
   <si>
     <t>Efectivo</t>
+  </si>
+  <si>
+    <t>01/02/2026</t>
+  </si>
+  <si>
+    <t>Sueldo febrero</t>
+  </si>
+  <si>
+    <t>Ingreso</t>
+  </si>
+  <si>
+    <t>Finanzas</t>
+  </si>
+  <si>
+    <t>Transferencia</t>
   </si>
 </sst>
 </file>
@@ -473,17 +494,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F502"/>
+  <dimension ref="A1:G502"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" defaultColWidth="18"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" ht="40" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -492,8 +514,9 @@
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
-    </row>
-    <row r="2" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="1"/>
+    </row>
+    <row r="2" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -512,1562 +535,1597 @@
       <c r="F2" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3" s="4">
         <v>45.5</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B4" s="4">
         <v>12</v>
       </c>
       <c r="C4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="4">
+        <v>4500</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="5"/>
-    </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" s="5"/>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" s="5"/>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="5"/>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B9" s="5"/>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B10" s="5"/>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B11" s="5"/>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B12" s="5"/>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B13" s="5"/>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B14" s="5"/>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B15" s="5"/>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B16" s="5"/>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="5"/>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="5"/>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B19" s="5"/>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="5"/>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B21" s="5"/>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B22" s="5"/>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B23" s="5"/>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B24" s="5"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B25" s="5"/>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B26" s="5"/>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B27" s="5"/>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B28" s="5"/>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B29" s="5"/>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B30" s="5"/>
     </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B31" s="5"/>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B32" s="5"/>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B33" s="5"/>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B34" s="5"/>
     </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B35" s="5"/>
     </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B36" s="5"/>
     </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B37" s="5"/>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B38" s="5"/>
     </row>
-    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B39" s="5"/>
     </row>
-    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B40" s="5"/>
     </row>
-    <row r="41" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B41" s="5"/>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B42" s="5"/>
     </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B43" s="5"/>
     </row>
-    <row r="44" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B44" s="5"/>
     </row>
-    <row r="45" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B45" s="5"/>
     </row>
-    <row r="46" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B46" s="5"/>
     </row>
-    <row r="47" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B47" s="5"/>
     </row>
-    <row r="48" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B48" s="5"/>
     </row>
-    <row r="49" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B49" s="5"/>
     </row>
-    <row r="50" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B50" s="5"/>
     </row>
-    <row r="51" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B51" s="5"/>
     </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B52" s="5"/>
     </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B53" s="5"/>
     </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B54" s="5"/>
     </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B55" s="5"/>
     </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B56" s="5"/>
     </row>
-    <row r="57" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B57" s="5"/>
     </row>
-    <row r="58" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B58" s="5"/>
     </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B59" s="5"/>
     </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B60" s="5"/>
     </row>
-    <row r="61" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B61" s="5"/>
     </row>
-    <row r="62" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B62" s="5"/>
     </row>
-    <row r="63" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B63" s="5"/>
     </row>
-    <row r="64" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B64" s="5"/>
     </row>
-    <row r="65" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B65" s="5"/>
     </row>
-    <row r="66" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B66" s="5"/>
     </row>
-    <row r="67" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B67" s="5"/>
     </row>
-    <row r="68" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B68" s="5"/>
     </row>
-    <row r="69" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B69" s="5"/>
     </row>
-    <row r="70" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B70" s="5"/>
     </row>
-    <row r="71" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B71" s="5"/>
     </row>
-    <row r="72" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B72" s="5"/>
     </row>
-    <row r="73" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B73" s="5"/>
     </row>
-    <row r="74" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B74" s="5"/>
     </row>
-    <row r="75" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B75" s="5"/>
     </row>
-    <row r="76" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B76" s="5"/>
     </row>
-    <row r="77" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B77" s="5"/>
     </row>
-    <row r="78" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B78" s="5"/>
     </row>
-    <row r="79" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B79" s="5"/>
     </row>
-    <row r="80" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B80" s="5"/>
     </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B81" s="5"/>
     </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B82" s="5"/>
     </row>
-    <row r="83" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B83" s="5"/>
     </row>
-    <row r="84" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B84" s="5"/>
     </row>
-    <row r="85" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B85" s="5"/>
     </row>
-    <row r="86" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B86" s="5"/>
     </row>
-    <row r="87" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B87" s="5"/>
     </row>
-    <row r="88" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B88" s="5"/>
     </row>
-    <row r="89" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B89" s="5"/>
     </row>
-    <row r="90" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B90" s="5"/>
     </row>
-    <row r="91" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B91" s="5"/>
     </row>
-    <row r="92" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B92" s="5"/>
     </row>
-    <row r="93" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B93" s="5"/>
     </row>
-    <row r="94" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B94" s="5"/>
     </row>
-    <row r="95" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B95" s="5"/>
     </row>
-    <row r="96" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B96" s="5"/>
     </row>
-    <row r="97" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B97" s="5"/>
     </row>
-    <row r="98" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B98" s="5"/>
     </row>
-    <row r="99" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B99" s="5"/>
     </row>
-    <row r="100" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B100" s="5"/>
     </row>
-    <row r="101" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B101" s="5"/>
     </row>
-    <row r="102" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B102" s="5"/>
     </row>
-    <row r="103" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B103" s="5"/>
     </row>
-    <row r="104" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B104" s="5"/>
     </row>
-    <row r="105" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B105" s="5"/>
     </row>
-    <row r="106" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B106" s="5"/>
     </row>
-    <row r="107" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B107" s="5"/>
     </row>
-    <row r="108" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B108" s="5"/>
     </row>
-    <row r="109" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B109" s="5"/>
     </row>
-    <row r="110" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B110" s="5"/>
     </row>
-    <row r="111" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B111" s="5"/>
     </row>
-    <row r="112" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B112" s="5"/>
     </row>
-    <row r="113" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B113" s="5"/>
     </row>
-    <row r="114" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B114" s="5"/>
     </row>
-    <row r="115" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B115" s="5"/>
     </row>
-    <row r="116" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B116" s="5"/>
     </row>
-    <row r="117" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B117" s="5"/>
     </row>
-    <row r="118" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B118" s="5"/>
     </row>
-    <row r="119" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B119" s="5"/>
     </row>
-    <row r="120" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B120" s="5"/>
     </row>
-    <row r="121" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B121" s="5"/>
     </row>
-    <row r="122" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B122" s="5"/>
     </row>
-    <row r="123" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B123" s="5"/>
     </row>
-    <row r="124" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B124" s="5"/>
     </row>
-    <row r="125" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="125" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B125" s="5"/>
     </row>
-    <row r="126" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="126" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B126" s="5"/>
     </row>
-    <row r="127" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="127" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B127" s="5"/>
     </row>
-    <row r="128" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="128" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B128" s="5"/>
     </row>
-    <row r="129" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="129" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B129" s="5"/>
     </row>
-    <row r="130" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="130" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B130" s="5"/>
     </row>
-    <row r="131" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="131" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B131" s="5"/>
     </row>
-    <row r="132" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="132" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B132" s="5"/>
     </row>
-    <row r="133" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="133" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B133" s="5"/>
     </row>
-    <row r="134" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="134" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B134" s="5"/>
     </row>
-    <row r="135" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="135" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B135" s="5"/>
     </row>
-    <row r="136" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="136" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B136" s="5"/>
     </row>
-    <row r="137" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="137" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B137" s="5"/>
     </row>
-    <row r="138" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="138" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B138" s="5"/>
     </row>
-    <row r="139" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="139" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B139" s="5"/>
     </row>
-    <row r="140" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="140" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B140" s="5"/>
     </row>
-    <row r="141" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="141" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B141" s="5"/>
     </row>
-    <row r="142" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="142" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B142" s="5"/>
     </row>
-    <row r="143" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="143" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B143" s="5"/>
     </row>
-    <row r="144" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="144" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B144" s="5"/>
     </row>
-    <row r="145" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="145" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B145" s="5"/>
     </row>
-    <row r="146" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="146" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B146" s="5"/>
     </row>
-    <row r="147" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="147" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B147" s="5"/>
     </row>
-    <row r="148" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="148" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B148" s="5"/>
     </row>
-    <row r="149" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="149" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B149" s="5"/>
     </row>
-    <row r="150" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="150" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B150" s="5"/>
     </row>
-    <row r="151" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="151" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B151" s="5"/>
     </row>
-    <row r="152" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="152" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B152" s="5"/>
     </row>
-    <row r="153" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="153" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B153" s="5"/>
     </row>
-    <row r="154" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="154" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B154" s="5"/>
     </row>
-    <row r="155" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="155" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B155" s="5"/>
     </row>
-    <row r="156" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="156" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B156" s="5"/>
     </row>
-    <row r="157" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="157" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B157" s="5"/>
     </row>
-    <row r="158" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="158" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B158" s="5"/>
     </row>
-    <row r="159" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="159" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B159" s="5"/>
     </row>
-    <row r="160" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="160" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B160" s="5"/>
     </row>
-    <row r="161" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="161" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B161" s="5"/>
     </row>
-    <row r="162" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="162" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B162" s="5"/>
     </row>
-    <row r="163" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="163" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B163" s="5"/>
     </row>
-    <row r="164" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="164" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B164" s="5"/>
     </row>
-    <row r="165" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="165" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B165" s="5"/>
     </row>
-    <row r="166" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="166" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B166" s="5"/>
     </row>
-    <row r="167" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="167" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B167" s="5"/>
     </row>
-    <row r="168" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="168" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B168" s="5"/>
     </row>
-    <row r="169" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="169" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B169" s="5"/>
     </row>
-    <row r="170" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="170" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B170" s="5"/>
     </row>
-    <row r="171" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="171" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B171" s="5"/>
     </row>
-    <row r="172" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="172" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B172" s="5"/>
     </row>
-    <row r="173" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="173" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B173" s="5"/>
     </row>
-    <row r="174" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="174" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B174" s="5"/>
     </row>
-    <row r="175" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="175" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B175" s="5"/>
     </row>
-    <row r="176" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="176" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B176" s="5"/>
     </row>
-    <row r="177" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="177" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B177" s="5"/>
     </row>
-    <row r="178" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="178" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B178" s="5"/>
     </row>
-    <row r="179" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="179" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B179" s="5"/>
     </row>
-    <row r="180" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="180" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B180" s="5"/>
     </row>
-    <row r="181" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="181" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B181" s="5"/>
     </row>
-    <row r="182" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="182" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B182" s="5"/>
     </row>
-    <row r="183" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="183" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B183" s="5"/>
     </row>
-    <row r="184" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="184" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B184" s="5"/>
     </row>
-    <row r="185" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="185" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B185" s="5"/>
     </row>
-    <row r="186" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="186" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B186" s="5"/>
     </row>
-    <row r="187" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="187" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B187" s="5"/>
     </row>
-    <row r="188" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="188" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B188" s="5"/>
     </row>
-    <row r="189" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="189" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B189" s="5"/>
     </row>
-    <row r="190" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="190" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B190" s="5"/>
     </row>
-    <row r="191" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="191" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B191" s="5"/>
     </row>
-    <row r="192" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="192" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B192" s="5"/>
     </row>
-    <row r="193" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="193" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B193" s="5"/>
     </row>
-    <row r="194" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="194" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B194" s="5"/>
     </row>
-    <row r="195" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="195" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B195" s="5"/>
     </row>
-    <row r="196" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="196" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B196" s="5"/>
     </row>
-    <row r="197" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="197" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B197" s="5"/>
     </row>
-    <row r="198" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="198" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B198" s="5"/>
     </row>
-    <row r="199" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="199" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B199" s="5"/>
     </row>
-    <row r="200" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="200" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B200" s="5"/>
     </row>
-    <row r="201" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="201" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B201" s="5"/>
     </row>
-    <row r="202" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="202" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B202" s="5"/>
     </row>
-    <row r="203" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="203" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B203" s="5"/>
     </row>
-    <row r="204" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="204" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B204" s="5"/>
     </row>
-    <row r="205" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="205" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B205" s="5"/>
     </row>
-    <row r="206" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="206" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B206" s="5"/>
     </row>
-    <row r="207" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="207" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B207" s="5"/>
     </row>
-    <row r="208" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="208" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B208" s="5"/>
     </row>
-    <row r="209" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="209" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B209" s="5"/>
     </row>
-    <row r="210" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="210" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B210" s="5"/>
     </row>
-    <row r="211" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="211" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B211" s="5"/>
     </row>
-    <row r="212" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="212" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B212" s="5"/>
     </row>
-    <row r="213" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="213" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B213" s="5"/>
     </row>
-    <row r="214" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="214" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B214" s="5"/>
     </row>
-    <row r="215" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="215" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B215" s="5"/>
     </row>
-    <row r="216" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="216" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B216" s="5"/>
     </row>
-    <row r="217" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="217" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B217" s="5"/>
     </row>
-    <row r="218" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="218" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B218" s="5"/>
     </row>
-    <row r="219" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="219" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B219" s="5"/>
     </row>
-    <row r="220" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="220" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B220" s="5"/>
     </row>
-    <row r="221" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="221" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B221" s="5"/>
     </row>
-    <row r="222" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="222" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B222" s="5"/>
     </row>
-    <row r="223" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="223" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B223" s="5"/>
     </row>
-    <row r="224" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="224" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B224" s="5"/>
     </row>
-    <row r="225" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="225" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B225" s="5"/>
     </row>
-    <row r="226" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="226" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B226" s="5"/>
     </row>
-    <row r="227" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="227" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B227" s="5"/>
     </row>
-    <row r="228" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="228" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B228" s="5"/>
     </row>
-    <row r="229" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="229" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B229" s="5"/>
     </row>
-    <row r="230" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="230" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B230" s="5"/>
     </row>
-    <row r="231" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="231" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B231" s="5"/>
     </row>
-    <row r="232" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="232" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B232" s="5"/>
     </row>
-    <row r="233" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="233" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B233" s="5"/>
     </row>
-    <row r="234" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="234" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B234" s="5"/>
     </row>
-    <row r="235" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="235" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B235" s="5"/>
     </row>
-    <row r="236" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="236" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B236" s="5"/>
     </row>
-    <row r="237" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="237" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B237" s="5"/>
     </row>
-    <row r="238" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="238" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B238" s="5"/>
     </row>
-    <row r="239" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="239" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B239" s="5"/>
     </row>
-    <row r="240" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="240" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B240" s="5"/>
     </row>
-    <row r="241" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="241" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B241" s="5"/>
     </row>
-    <row r="242" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="242" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B242" s="5"/>
     </row>
-    <row r="243" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="243" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B243" s="5"/>
     </row>
-    <row r="244" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="244" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B244" s="5"/>
     </row>
-    <row r="245" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="245" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B245" s="5"/>
     </row>
-    <row r="246" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="246" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B246" s="5"/>
     </row>
-    <row r="247" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="247" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B247" s="5"/>
     </row>
-    <row r="248" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="248" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B248" s="5"/>
     </row>
-    <row r="249" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="249" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B249" s="5"/>
     </row>
-    <row r="250" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="250" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B250" s="5"/>
     </row>
-    <row r="251" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="251" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B251" s="5"/>
     </row>
-    <row r="252" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="252" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B252" s="5"/>
     </row>
-    <row r="253" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="253" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B253" s="5"/>
     </row>
-    <row r="254" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="254" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B254" s="5"/>
     </row>
-    <row r="255" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="255" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B255" s="5"/>
     </row>
-    <row r="256" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="256" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B256" s="5"/>
     </row>
-    <row r="257" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="257" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B257" s="5"/>
     </row>
-    <row r="258" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="258" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B258" s="5"/>
     </row>
-    <row r="259" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="259" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B259" s="5"/>
     </row>
-    <row r="260" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="260" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B260" s="5"/>
     </row>
-    <row r="261" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="261" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B261" s="5"/>
     </row>
-    <row r="262" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="262" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B262" s="5"/>
     </row>
-    <row r="263" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="263" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B263" s="5"/>
     </row>
-    <row r="264" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="264" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B264" s="5"/>
     </row>
-    <row r="265" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="265" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B265" s="5"/>
     </row>
-    <row r="266" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="266" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B266" s="5"/>
     </row>
-    <row r="267" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="267" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B267" s="5"/>
     </row>
-    <row r="268" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="268" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B268" s="5"/>
     </row>
-    <row r="269" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="269" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B269" s="5"/>
     </row>
-    <row r="270" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="270" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B270" s="5"/>
     </row>
-    <row r="271" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="271" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B271" s="5"/>
     </row>
-    <row r="272" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="272" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B272" s="5"/>
     </row>
-    <row r="273" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="273" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B273" s="5"/>
     </row>
-    <row r="274" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="274" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B274" s="5"/>
     </row>
-    <row r="275" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="275" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B275" s="5"/>
     </row>
-    <row r="276" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="276" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B276" s="5"/>
     </row>
-    <row r="277" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="277" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B277" s="5"/>
     </row>
-    <row r="278" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="278" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B278" s="5"/>
     </row>
-    <row r="279" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="279" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B279" s="5"/>
     </row>
-    <row r="280" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="280" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B280" s="5"/>
     </row>
-    <row r="281" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="281" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B281" s="5"/>
     </row>
-    <row r="282" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="282" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B282" s="5"/>
     </row>
-    <row r="283" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="283" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B283" s="5"/>
     </row>
-    <row r="284" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="284" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B284" s="5"/>
     </row>
-    <row r="285" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="285" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B285" s="5"/>
     </row>
-    <row r="286" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="286" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B286" s="5"/>
     </row>
-    <row r="287" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="287" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B287" s="5"/>
     </row>
-    <row r="288" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="288" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B288" s="5"/>
     </row>
-    <row r="289" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="289" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B289" s="5"/>
     </row>
-    <row r="290" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="290" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B290" s="5"/>
     </row>
-    <row r="291" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="291" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B291" s="5"/>
     </row>
-    <row r="292" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="292" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B292" s="5"/>
     </row>
-    <row r="293" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="293" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B293" s="5"/>
     </row>
-    <row r="294" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="294" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B294" s="5"/>
     </row>
-    <row r="295" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="295" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B295" s="5"/>
     </row>
-    <row r="296" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="296" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B296" s="5"/>
     </row>
-    <row r="297" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="297" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B297" s="5"/>
     </row>
-    <row r="298" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="298" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B298" s="5"/>
     </row>
-    <row r="299" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="299" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B299" s="5"/>
     </row>
-    <row r="300" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="300" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B300" s="5"/>
     </row>
-    <row r="301" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="301" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B301" s="5"/>
     </row>
-    <row r="302" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="302" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B302" s="5"/>
     </row>
-    <row r="303" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="303" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B303" s="5"/>
     </row>
-    <row r="304" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="304" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B304" s="5"/>
     </row>
-    <row r="305" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="305" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B305" s="5"/>
     </row>
-    <row r="306" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="306" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B306" s="5"/>
     </row>
-    <row r="307" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="307" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B307" s="5"/>
     </row>
-    <row r="308" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="308" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B308" s="5"/>
     </row>
-    <row r="309" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="309" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B309" s="5"/>
     </row>
-    <row r="310" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="310" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B310" s="5"/>
     </row>
-    <row r="311" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="311" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B311" s="5"/>
     </row>
-    <row r="312" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="312" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B312" s="5"/>
     </row>
-    <row r="313" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="313" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B313" s="5"/>
     </row>
-    <row r="314" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="314" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B314" s="5"/>
     </row>
-    <row r="315" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="315" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B315" s="5"/>
     </row>
-    <row r="316" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="316" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B316" s="5"/>
     </row>
-    <row r="317" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="317" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B317" s="5"/>
     </row>
-    <row r="318" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="318" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B318" s="5"/>
     </row>
-    <row r="319" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="319" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B319" s="5"/>
     </row>
-    <row r="320" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="320" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B320" s="5"/>
     </row>
-    <row r="321" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="321" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B321" s="5"/>
     </row>
-    <row r="322" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="322" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B322" s="5"/>
     </row>
-    <row r="323" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="323" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B323" s="5"/>
     </row>
-    <row r="324" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="324" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B324" s="5"/>
     </row>
-    <row r="325" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="325" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B325" s="5"/>
     </row>
-    <row r="326" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="326" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B326" s="5"/>
     </row>
-    <row r="327" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="327" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B327" s="5"/>
     </row>
-    <row r="328" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="328" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B328" s="5"/>
     </row>
-    <row r="329" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="329" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B329" s="5"/>
     </row>
-    <row r="330" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="330" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B330" s="5"/>
     </row>
-    <row r="331" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="331" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B331" s="5"/>
     </row>
-    <row r="332" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="332" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B332" s="5"/>
     </row>
-    <row r="333" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="333" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B333" s="5"/>
     </row>
-    <row r="334" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="334" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B334" s="5"/>
     </row>
-    <row r="335" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="335" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B335" s="5"/>
     </row>
-    <row r="336" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="336" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B336" s="5"/>
     </row>
-    <row r="337" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="337" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B337" s="5"/>
     </row>
-    <row r="338" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="338" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B338" s="5"/>
     </row>
-    <row r="339" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="339" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B339" s="5"/>
     </row>
-    <row r="340" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="340" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B340" s="5"/>
     </row>
-    <row r="341" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="341" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B341" s="5"/>
     </row>
-    <row r="342" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="342" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B342" s="5"/>
     </row>
-    <row r="343" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="343" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B343" s="5"/>
     </row>
-    <row r="344" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="344" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B344" s="5"/>
     </row>
-    <row r="345" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="345" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B345" s="5"/>
     </row>
-    <row r="346" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="346" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B346" s="5"/>
     </row>
-    <row r="347" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="347" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B347" s="5"/>
     </row>
-    <row r="348" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="348" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B348" s="5"/>
     </row>
-    <row r="349" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="349" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B349" s="5"/>
     </row>
-    <row r="350" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="350" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B350" s="5"/>
     </row>
-    <row r="351" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="351" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B351" s="5"/>
     </row>
-    <row r="352" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="352" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B352" s="5"/>
     </row>
-    <row r="353" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="353" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B353" s="5"/>
     </row>
-    <row r="354" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="354" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B354" s="5"/>
     </row>
-    <row r="355" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="355" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B355" s="5"/>
     </row>
-    <row r="356" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="356" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B356" s="5"/>
     </row>
-    <row r="357" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="357" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B357" s="5"/>
     </row>
-    <row r="358" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="358" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B358" s="5"/>
     </row>
-    <row r="359" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="359" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B359" s="5"/>
     </row>
-    <row r="360" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="360" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B360" s="5"/>
     </row>
-    <row r="361" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="361" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B361" s="5"/>
     </row>
-    <row r="362" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="362" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B362" s="5"/>
     </row>
-    <row r="363" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="363" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B363" s="5"/>
     </row>
-    <row r="364" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="364" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B364" s="5"/>
     </row>
-    <row r="365" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="365" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B365" s="5"/>
     </row>
-    <row r="366" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="366" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B366" s="5"/>
     </row>
-    <row r="367" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="367" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B367" s="5"/>
     </row>
-    <row r="368" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="368" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B368" s="5"/>
     </row>
-    <row r="369" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="369" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B369" s="5"/>
     </row>
-    <row r="370" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="370" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B370" s="5"/>
     </row>
-    <row r="371" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="371" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B371" s="5"/>
     </row>
-    <row r="372" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="372" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B372" s="5"/>
     </row>
-    <row r="373" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="373" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B373" s="5"/>
     </row>
-    <row r="374" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="374" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B374" s="5"/>
     </row>
-    <row r="375" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="375" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B375" s="5"/>
     </row>
-    <row r="376" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="376" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B376" s="5"/>
     </row>
-    <row r="377" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="377" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B377" s="5"/>
     </row>
-    <row r="378" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="378" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B378" s="5"/>
     </row>
-    <row r="379" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="379" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B379" s="5"/>
     </row>
-    <row r="380" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="380" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B380" s="5"/>
     </row>
-    <row r="381" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="381" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B381" s="5"/>
     </row>
-    <row r="382" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="382" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B382" s="5"/>
     </row>
-    <row r="383" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="383" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B383" s="5"/>
     </row>
-    <row r="384" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="384" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B384" s="5"/>
     </row>
-    <row r="385" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="385" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B385" s="5"/>
     </row>
-    <row r="386" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="386" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B386" s="5"/>
     </row>
-    <row r="387" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="387" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B387" s="5"/>
     </row>
-    <row r="388" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="388" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B388" s="5"/>
     </row>
-    <row r="389" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="389" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B389" s="5"/>
     </row>
-    <row r="390" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="390" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B390" s="5"/>
     </row>
-    <row r="391" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="391" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B391" s="5"/>
     </row>
-    <row r="392" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="392" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B392" s="5"/>
     </row>
-    <row r="393" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="393" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B393" s="5"/>
     </row>
-    <row r="394" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="394" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B394" s="5"/>
     </row>
-    <row r="395" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="395" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B395" s="5"/>
     </row>
-    <row r="396" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="396" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B396" s="5"/>
     </row>
-    <row r="397" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="397" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B397" s="5"/>
     </row>
-    <row r="398" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="398" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B398" s="5"/>
     </row>
-    <row r="399" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="399" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B399" s="5"/>
     </row>
-    <row r="400" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="400" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B400" s="5"/>
     </row>
-    <row r="401" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="401" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B401" s="5"/>
     </row>
-    <row r="402" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="402" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B402" s="5"/>
     </row>
-    <row r="403" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="403" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B403" s="5"/>
     </row>
-    <row r="404" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="404" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B404" s="5"/>
     </row>
-    <row r="405" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="405" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B405" s="5"/>
     </row>
-    <row r="406" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="406" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B406" s="5"/>
     </row>
-    <row r="407" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="407" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B407" s="5"/>
     </row>
-    <row r="408" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="408" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B408" s="5"/>
     </row>
-    <row r="409" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="409" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B409" s="5"/>
     </row>
-    <row r="410" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="410" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B410" s="5"/>
     </row>
-    <row r="411" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="411" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B411" s="5"/>
     </row>
-    <row r="412" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="412" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B412" s="5"/>
     </row>
-    <row r="413" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="413" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B413" s="5"/>
     </row>
-    <row r="414" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="414" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B414" s="5"/>
     </row>
-    <row r="415" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="415" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B415" s="5"/>
     </row>
-    <row r="416" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="416" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B416" s="5"/>
     </row>
-    <row r="417" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="417" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B417" s="5"/>
     </row>
-    <row r="418" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="418" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B418" s="5"/>
     </row>
-    <row r="419" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="419" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B419" s="5"/>
     </row>
-    <row r="420" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="420" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B420" s="5"/>
     </row>
-    <row r="421" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="421" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B421" s="5"/>
     </row>
-    <row r="422" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="422" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B422" s="5"/>
     </row>
-    <row r="423" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="423" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B423" s="5"/>
     </row>
-    <row r="424" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="424" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B424" s="5"/>
     </row>
-    <row r="425" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="425" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B425" s="5"/>
     </row>
-    <row r="426" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="426" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B426" s="5"/>
     </row>
-    <row r="427" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="427" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B427" s="5"/>
     </row>
-    <row r="428" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="428" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B428" s="5"/>
     </row>
-    <row r="429" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="429" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B429" s="5"/>
     </row>
-    <row r="430" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="430" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B430" s="5"/>
     </row>
-    <row r="431" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="431" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B431" s="5"/>
     </row>
-    <row r="432" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="432" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B432" s="5"/>
     </row>
-    <row r="433" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="433" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B433" s="5"/>
     </row>
-    <row r="434" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="434" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B434" s="5"/>
     </row>
-    <row r="435" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="435" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B435" s="5"/>
     </row>
-    <row r="436" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="436" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B436" s="5"/>
     </row>
-    <row r="437" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="437" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B437" s="5"/>
     </row>
-    <row r="438" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="438" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B438" s="5"/>
     </row>
-    <row r="439" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="439" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B439" s="5"/>
     </row>
-    <row r="440" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="440" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B440" s="5"/>
     </row>
-    <row r="441" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="441" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B441" s="5"/>
     </row>
-    <row r="442" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="442" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B442" s="5"/>
     </row>
-    <row r="443" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="443" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B443" s="5"/>
     </row>
-    <row r="444" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="444" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B444" s="5"/>
     </row>
-    <row r="445" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="445" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B445" s="5"/>
     </row>
-    <row r="446" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="446" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B446" s="5"/>
     </row>
-    <row r="447" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="447" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B447" s="5"/>
     </row>
-    <row r="448" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="448" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B448" s="5"/>
     </row>
-    <row r="449" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="449" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B449" s="5"/>
     </row>
-    <row r="450" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="450" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B450" s="5"/>
     </row>
-    <row r="451" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="451" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B451" s="5"/>
     </row>
-    <row r="452" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="452" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B452" s="5"/>
     </row>
-    <row r="453" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="453" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B453" s="5"/>
     </row>
-    <row r="454" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="454" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B454" s="5"/>
     </row>
-    <row r="455" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="455" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B455" s="5"/>
     </row>
-    <row r="456" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="456" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B456" s="5"/>
     </row>
-    <row r="457" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="457" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B457" s="5"/>
     </row>
-    <row r="458" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="458" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B458" s="5"/>
     </row>
-    <row r="459" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="459" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B459" s="5"/>
     </row>
-    <row r="460" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="460" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B460" s="5"/>
     </row>
-    <row r="461" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="461" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B461" s="5"/>
     </row>
-    <row r="462" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="462" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B462" s="5"/>
     </row>
-    <row r="463" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="463" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B463" s="5"/>
     </row>
-    <row r="464" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="464" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B464" s="5"/>
     </row>
-    <row r="465" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="465" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B465" s="5"/>
     </row>
-    <row r="466" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="466" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B466" s="5"/>
     </row>
-    <row r="467" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="467" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B467" s="5"/>
     </row>
-    <row r="468" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="468" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B468" s="5"/>
     </row>
-    <row r="469" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="469" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B469" s="5"/>
     </row>
-    <row r="470" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="470" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B470" s="5"/>
     </row>
-    <row r="471" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="471" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B471" s="5"/>
     </row>
-    <row r="472" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="472" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B472" s="5"/>
     </row>
-    <row r="473" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="473" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B473" s="5"/>
     </row>
-    <row r="474" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="474" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B474" s="5"/>
     </row>
-    <row r="475" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="475" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B475" s="5"/>
     </row>
-    <row r="476" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="476" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B476" s="5"/>
     </row>
-    <row r="477" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="477" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B477" s="5"/>
     </row>
-    <row r="478" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="478" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B478" s="5"/>
     </row>
-    <row r="479" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="479" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B479" s="5"/>
     </row>
-    <row r="480" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="480" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B480" s="5"/>
     </row>
-    <row r="481" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="481" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B481" s="5"/>
     </row>
-    <row r="482" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="482" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B482" s="5"/>
     </row>
-    <row r="483" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="483" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B483" s="5"/>
     </row>
-    <row r="484" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="484" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B484" s="5"/>
     </row>
-    <row r="485" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="485" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B485" s="5"/>
     </row>
-    <row r="486" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="486" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B486" s="5"/>
     </row>
-    <row r="487" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="487" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B487" s="5"/>
     </row>
-    <row r="488" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="488" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B488" s="5"/>
     </row>
-    <row r="489" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="489" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B489" s="5"/>
     </row>
-    <row r="490" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="490" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B490" s="5"/>
     </row>
-    <row r="491" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="491" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B491" s="5"/>
     </row>
-    <row r="492" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="492" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B492" s="5"/>
     </row>
-    <row r="493" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="493" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B493" s="5"/>
     </row>
-    <row r="494" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="494" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B494" s="5"/>
     </row>
-    <row r="495" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="495" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B495" s="5"/>
     </row>
-    <row r="496" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="496" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B496" s="5"/>
     </row>
-    <row r="497" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="497" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B497" s="5"/>
     </row>
-    <row r="498" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="498" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B498" s="5"/>
     </row>
-    <row r="499" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="499" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B499" s="5"/>
     </row>
-    <row r="500" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="500" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B500" s="5"/>
     </row>
-    <row r="501" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="501" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B501" s="5"/>
     </row>
-    <row r="502" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="502" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B502" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Categoría inválida" error="Selecciona una categoría de la lista o déjala vacía para que NETO la asigne." sqref="D10:D502">
+  <dataValidations count="8">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Tipo inválido" error="Selecciona Gasto o Ingreso. Si lo dejas vacío, NETO lo asume como Gasto." sqref="D10:D502">
+      <formula1>"Gasto,Ingreso"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Tipo inválido" error="Selecciona Gasto o Ingreso. Si lo dejas vacío, NETO lo asume como Gasto." sqref="D3:D502">
+      <formula1>"Gasto,Ingreso"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Categoría inválida" error="Selecciona una categoría de la lista o déjala vacía para que NETO la asigne." sqref="E10:E502">
       <formula1>"Alimentación,Transporte,Vivienda,Salud,Entretenimiento,Compras,Educación,Finanzas,Trabajo_Negocio,Otros"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Categoría inválida" error="Selecciona una categoría de la lista o déjala vacía para que NETO la asigne." sqref="D3:D502">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Categoría inválida" error="Selecciona una categoría de la lista o déjala vacía para que NETO la asigne." sqref="E3:E502">
       <formula1>"Alimentación,Transporte,Vivienda,Salud,Entretenimiento,Compras,Educación,Finanzas,Trabajo_Negocio,Otros"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="E10:E502">
+    <dataValidation type="list" allowBlank="1" sqref="F10:F502">
       <formula1>"Yape,Plin,Débito,Crédito,Efectivo,Transferencia,Otro"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="E3:E502">
+    <dataValidation type="list" allowBlank="1" sqref="F3:F502">
       <formula1>"Yape,Plin,Débito,Crédito,Efectivo,Transferencia,Otro"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="F10:F502">
+    <dataValidation type="list" allowBlank="1" sqref="G10:G502">
       <formula1>"BCP,Interbank,BBVA,Scotiabank,Yape,Plin,Otro"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="F3:F502">
+    <dataValidation type="list" allowBlank="1" sqref="G3:G502">
       <formula1>"BCP,Interbank,BBVA,Scotiabank,Yape,Plin,Otro"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: agregar columna Subcategoría a plantilla Excel y handler
- Plantilla ahora tiene 8 columnas: Fecha, Monto, Comercio, Tipo, Categoría, Subcategoría, Método, Banco
- Dropdown de validación con todas las subcategorías del árbol canónico de NETO
- Handler auto-detecta 3 formatos (6, 7 u 8 columnas) para retrocompatibilidad
- GPT categoriza filas sin categoría Y sin subcategoría

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantilla_gastos.xlsx
+++ b/public/plantilla_gastos.xlsx
@@ -11,9 +11,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
-  <si>
-    <t>PLANTILLA NETO — Carga de Gastos e Ingresos Históricos. Completa cada fila con un movimiento. Las columnas Tipo, Categoría, Método de Pago y Banco son opcionales (NETO las asigna automáticamente con IA).</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
+  <si>
+    <t>PLANTILLA NETO — Carga de Gastos e Ingresos Históricos. Completa cada fila con un movimiento. Tipo, Categoría, Subcategoría, Método de Pago y Banco son opcionales (NETO las asigna automáticamente con IA).</t>
   </si>
   <si>
     <t>Fecha</t>
@@ -31,6 +31,9 @@
     <t>Categoría</t>
   </si>
   <si>
+    <t>Subcategoría</t>
+  </si>
+  <si>
     <t>Método de Pago</t>
   </si>
   <si>
@@ -49,6 +52,9 @@
     <t>Alimentación</t>
   </si>
   <si>
+    <t>supermercado</t>
+  </si>
+  <si>
     <t>Yape</t>
   </si>
   <si>
@@ -61,10 +67,16 @@
     <t>Taxi al centro</t>
   </si>
   <si>
+    <t>Transporte</t>
+  </si>
+  <si>
+    <t>taxi</t>
+  </si>
+  <si>
+    <t>Efectivo</t>
+  </si>
+  <si>
     <t/>
-  </si>
-  <si>
-    <t>Efectivo</t>
   </si>
   <si>
     <t>01/02/2026</t>
@@ -494,18 +506,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G502"/>
+  <dimension ref="A1:H502"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" defaultColWidth="18"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="5" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" ht="40" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -515,8 +527,9 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-    </row>
-    <row r="2" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -538,1572 +551,1584 @@
       <c r="G2" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H2" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B3" s="4">
         <v>45.5</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B4" s="4">
         <v>12</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B5" s="4">
         <v>4500</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="E5" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>22</v>
-      </c>
       <c r="G5" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="5"/>
     </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="5"/>
     </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="5"/>
     </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B9" s="5"/>
     </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" s="5"/>
     </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B11" s="5"/>
     </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B12" s="5"/>
     </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B13" s="5"/>
     </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B14" s="5"/>
     </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B15" s="5"/>
     </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B16" s="5"/>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B17" s="5"/>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B18" s="5"/>
     </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B19" s="5"/>
     </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B20" s="5"/>
     </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B21" s="5"/>
     </row>
-    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B22" s="5"/>
     </row>
-    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B23" s="5"/>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B24" s="5"/>
     </row>
-    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B25" s="5"/>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B26" s="5"/>
     </row>
-    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B27" s="5"/>
     </row>
-    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B28" s="5"/>
     </row>
-    <row r="29" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B29" s="5"/>
     </row>
-    <row r="30" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B30" s="5"/>
     </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B31" s="5"/>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B32" s="5"/>
     </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B33" s="5"/>
     </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B34" s="5"/>
     </row>
-    <row r="35" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B35" s="5"/>
     </row>
-    <row r="36" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B36" s="5"/>
     </row>
-    <row r="37" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B37" s="5"/>
     </row>
-    <row r="38" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B38" s="5"/>
     </row>
-    <row r="39" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B39" s="5"/>
     </row>
-    <row r="40" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B40" s="5"/>
     </row>
-    <row r="41" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B41" s="5"/>
     </row>
-    <row r="42" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B42" s="5"/>
     </row>
-    <row r="43" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B43" s="5"/>
     </row>
-    <row r="44" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B44" s="5"/>
     </row>
-    <row r="45" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B45" s="5"/>
     </row>
-    <row r="46" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B46" s="5"/>
     </row>
-    <row r="47" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B47" s="5"/>
     </row>
-    <row r="48" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B48" s="5"/>
     </row>
-    <row r="49" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B49" s="5"/>
     </row>
-    <row r="50" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B50" s="5"/>
     </row>
-    <row r="51" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B51" s="5"/>
     </row>
-    <row r="52" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B52" s="5"/>
     </row>
-    <row r="53" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B53" s="5"/>
     </row>
-    <row r="54" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B54" s="5"/>
     </row>
-    <row r="55" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B55" s="5"/>
     </row>
-    <row r="56" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B56" s="5"/>
     </row>
-    <row r="57" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B57" s="5"/>
     </row>
-    <row r="58" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B58" s="5"/>
     </row>
-    <row r="59" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B59" s="5"/>
     </row>
-    <row r="60" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B60" s="5"/>
     </row>
-    <row r="61" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B61" s="5"/>
     </row>
-    <row r="62" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B62" s="5"/>
     </row>
-    <row r="63" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B63" s="5"/>
     </row>
-    <row r="64" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B64" s="5"/>
     </row>
-    <row r="65" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B65" s="5"/>
     </row>
-    <row r="66" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B66" s="5"/>
     </row>
-    <row r="67" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B67" s="5"/>
     </row>
-    <row r="68" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B68" s="5"/>
     </row>
-    <row r="69" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B69" s="5"/>
     </row>
-    <row r="70" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B70" s="5"/>
     </row>
-    <row r="71" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B71" s="5"/>
     </row>
-    <row r="72" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B72" s="5"/>
     </row>
-    <row r="73" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B73" s="5"/>
     </row>
-    <row r="74" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B74" s="5"/>
     </row>
-    <row r="75" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B75" s="5"/>
     </row>
-    <row r="76" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B76" s="5"/>
     </row>
-    <row r="77" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B77" s="5"/>
     </row>
-    <row r="78" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B78" s="5"/>
     </row>
-    <row r="79" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B79" s="5"/>
     </row>
-    <row r="80" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B80" s="5"/>
     </row>
-    <row r="81" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B81" s="5"/>
     </row>
-    <row r="82" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B82" s="5"/>
     </row>
-    <row r="83" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B83" s="5"/>
     </row>
-    <row r="84" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B84" s="5"/>
     </row>
-    <row r="85" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B85" s="5"/>
     </row>
-    <row r="86" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B86" s="5"/>
     </row>
-    <row r="87" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B87" s="5"/>
     </row>
-    <row r="88" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B88" s="5"/>
     </row>
-    <row r="89" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B89" s="5"/>
     </row>
-    <row r="90" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B90" s="5"/>
     </row>
-    <row r="91" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B91" s="5"/>
     </row>
-    <row r="92" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B92" s="5"/>
     </row>
-    <row r="93" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B93" s="5"/>
     </row>
-    <row r="94" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B94" s="5"/>
     </row>
-    <row r="95" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B95" s="5"/>
     </row>
-    <row r="96" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B96" s="5"/>
     </row>
-    <row r="97" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B97" s="5"/>
     </row>
-    <row r="98" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B98" s="5"/>
     </row>
-    <row r="99" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B99" s="5"/>
     </row>
-    <row r="100" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B100" s="5"/>
     </row>
-    <row r="101" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B101" s="5"/>
     </row>
-    <row r="102" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B102" s="5"/>
     </row>
-    <row r="103" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B103" s="5"/>
     </row>
-    <row r="104" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B104" s="5"/>
     </row>
-    <row r="105" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B105" s="5"/>
     </row>
-    <row r="106" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B106" s="5"/>
     </row>
-    <row r="107" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B107" s="5"/>
     </row>
-    <row r="108" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B108" s="5"/>
     </row>
-    <row r="109" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B109" s="5"/>
     </row>
-    <row r="110" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B110" s="5"/>
     </row>
-    <row r="111" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B111" s="5"/>
     </row>
-    <row r="112" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B112" s="5"/>
     </row>
-    <row r="113" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B113" s="5"/>
     </row>
-    <row r="114" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B114" s="5"/>
     </row>
-    <row r="115" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B115" s="5"/>
     </row>
-    <row r="116" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B116" s="5"/>
     </row>
-    <row r="117" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B117" s="5"/>
     </row>
-    <row r="118" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B118" s="5"/>
     </row>
-    <row r="119" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B119" s="5"/>
     </row>
-    <row r="120" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B120" s="5"/>
     </row>
-    <row r="121" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B121" s="5"/>
     </row>
-    <row r="122" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B122" s="5"/>
     </row>
-    <row r="123" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B123" s="5"/>
     </row>
-    <row r="124" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B124" s="5"/>
     </row>
-    <row r="125" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="125" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B125" s="5"/>
     </row>
-    <row r="126" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="126" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B126" s="5"/>
     </row>
-    <row r="127" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="127" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B127" s="5"/>
     </row>
-    <row r="128" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="128" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B128" s="5"/>
     </row>
-    <row r="129" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="129" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B129" s="5"/>
     </row>
-    <row r="130" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="130" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B130" s="5"/>
     </row>
-    <row r="131" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="131" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B131" s="5"/>
     </row>
-    <row r="132" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="132" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B132" s="5"/>
     </row>
-    <row r="133" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="133" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B133" s="5"/>
     </row>
-    <row r="134" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="134" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B134" s="5"/>
     </row>
-    <row r="135" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="135" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B135" s="5"/>
     </row>
-    <row r="136" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="136" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B136" s="5"/>
     </row>
-    <row r="137" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="137" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B137" s="5"/>
     </row>
-    <row r="138" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="138" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B138" s="5"/>
     </row>
-    <row r="139" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="139" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B139" s="5"/>
     </row>
-    <row r="140" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="140" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B140" s="5"/>
     </row>
-    <row r="141" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="141" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B141" s="5"/>
     </row>
-    <row r="142" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="142" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B142" s="5"/>
     </row>
-    <row r="143" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="143" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B143" s="5"/>
     </row>
-    <row r="144" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="144" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B144" s="5"/>
     </row>
-    <row r="145" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="145" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B145" s="5"/>
     </row>
-    <row r="146" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="146" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B146" s="5"/>
     </row>
-    <row r="147" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="147" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B147" s="5"/>
     </row>
-    <row r="148" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="148" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B148" s="5"/>
     </row>
-    <row r="149" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="149" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B149" s="5"/>
     </row>
-    <row r="150" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="150" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B150" s="5"/>
     </row>
-    <row r="151" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="151" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B151" s="5"/>
     </row>
-    <row r="152" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="152" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B152" s="5"/>
     </row>
-    <row r="153" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="153" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B153" s="5"/>
     </row>
-    <row r="154" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="154" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B154" s="5"/>
     </row>
-    <row r="155" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="155" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B155" s="5"/>
     </row>
-    <row r="156" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="156" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B156" s="5"/>
     </row>
-    <row r="157" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="157" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B157" s="5"/>
     </row>
-    <row r="158" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="158" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B158" s="5"/>
     </row>
-    <row r="159" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="159" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B159" s="5"/>
     </row>
-    <row r="160" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="160" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B160" s="5"/>
     </row>
-    <row r="161" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="161" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B161" s="5"/>
     </row>
-    <row r="162" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="162" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B162" s="5"/>
     </row>
-    <row r="163" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="163" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B163" s="5"/>
     </row>
-    <row r="164" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="164" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B164" s="5"/>
     </row>
-    <row r="165" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="165" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B165" s="5"/>
     </row>
-    <row r="166" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="166" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B166" s="5"/>
     </row>
-    <row r="167" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="167" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B167" s="5"/>
     </row>
-    <row r="168" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="168" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B168" s="5"/>
     </row>
-    <row r="169" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="169" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B169" s="5"/>
     </row>
-    <row r="170" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="170" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B170" s="5"/>
     </row>
-    <row r="171" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="171" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B171" s="5"/>
     </row>
-    <row r="172" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="172" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B172" s="5"/>
     </row>
-    <row r="173" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="173" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B173" s="5"/>
     </row>
-    <row r="174" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="174" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B174" s="5"/>
     </row>
-    <row r="175" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="175" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B175" s="5"/>
     </row>
-    <row r="176" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="176" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B176" s="5"/>
     </row>
-    <row r="177" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="177" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B177" s="5"/>
     </row>
-    <row r="178" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="178" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B178" s="5"/>
     </row>
-    <row r="179" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="179" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B179" s="5"/>
     </row>
-    <row r="180" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="180" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B180" s="5"/>
     </row>
-    <row r="181" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="181" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B181" s="5"/>
     </row>
-    <row r="182" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="182" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B182" s="5"/>
     </row>
-    <row r="183" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="183" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B183" s="5"/>
     </row>
-    <row r="184" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="184" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B184" s="5"/>
     </row>
-    <row r="185" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="185" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B185" s="5"/>
     </row>
-    <row r="186" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="186" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B186" s="5"/>
     </row>
-    <row r="187" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="187" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B187" s="5"/>
     </row>
-    <row r="188" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="188" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B188" s="5"/>
     </row>
-    <row r="189" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="189" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B189" s="5"/>
     </row>
-    <row r="190" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="190" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B190" s="5"/>
     </row>
-    <row r="191" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="191" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B191" s="5"/>
     </row>
-    <row r="192" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="192" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B192" s="5"/>
     </row>
-    <row r="193" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="193" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B193" s="5"/>
     </row>
-    <row r="194" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="194" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B194" s="5"/>
     </row>
-    <row r="195" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="195" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B195" s="5"/>
     </row>
-    <row r="196" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="196" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B196" s="5"/>
     </row>
-    <row r="197" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="197" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B197" s="5"/>
     </row>
-    <row r="198" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="198" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B198" s="5"/>
     </row>
-    <row r="199" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="199" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B199" s="5"/>
     </row>
-    <row r="200" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="200" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B200" s="5"/>
     </row>
-    <row r="201" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="201" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B201" s="5"/>
     </row>
-    <row r="202" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="202" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B202" s="5"/>
     </row>
-    <row r="203" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="203" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B203" s="5"/>
     </row>
-    <row r="204" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="204" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B204" s="5"/>
     </row>
-    <row r="205" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="205" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B205" s="5"/>
     </row>
-    <row r="206" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="206" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B206" s="5"/>
     </row>
-    <row r="207" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="207" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B207" s="5"/>
     </row>
-    <row r="208" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="208" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B208" s="5"/>
     </row>
-    <row r="209" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="209" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B209" s="5"/>
     </row>
-    <row r="210" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="210" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B210" s="5"/>
     </row>
-    <row r="211" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="211" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B211" s="5"/>
     </row>
-    <row r="212" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="212" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B212" s="5"/>
     </row>
-    <row r="213" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="213" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B213" s="5"/>
     </row>
-    <row r="214" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="214" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B214" s="5"/>
     </row>
-    <row r="215" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="215" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B215" s="5"/>
     </row>
-    <row r="216" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="216" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B216" s="5"/>
     </row>
-    <row r="217" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="217" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B217" s="5"/>
     </row>
-    <row r="218" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="218" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B218" s="5"/>
     </row>
-    <row r="219" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="219" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B219" s="5"/>
     </row>
-    <row r="220" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="220" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B220" s="5"/>
     </row>
-    <row r="221" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="221" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B221" s="5"/>
     </row>
-    <row r="222" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="222" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B222" s="5"/>
     </row>
-    <row r="223" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="223" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B223" s="5"/>
     </row>
-    <row r="224" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="224" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B224" s="5"/>
     </row>
-    <row r="225" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="225" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B225" s="5"/>
     </row>
-    <row r="226" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="226" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B226" s="5"/>
     </row>
-    <row r="227" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="227" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B227" s="5"/>
     </row>
-    <row r="228" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="228" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B228" s="5"/>
     </row>
-    <row r="229" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="229" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B229" s="5"/>
     </row>
-    <row r="230" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="230" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B230" s="5"/>
     </row>
-    <row r="231" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="231" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B231" s="5"/>
     </row>
-    <row r="232" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="232" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B232" s="5"/>
     </row>
-    <row r="233" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="233" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B233" s="5"/>
     </row>
-    <row r="234" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="234" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B234" s="5"/>
     </row>
-    <row r="235" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="235" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B235" s="5"/>
     </row>
-    <row r="236" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="236" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B236" s="5"/>
     </row>
-    <row r="237" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="237" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B237" s="5"/>
     </row>
-    <row r="238" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="238" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B238" s="5"/>
     </row>
-    <row r="239" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="239" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B239" s="5"/>
     </row>
-    <row r="240" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="240" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B240" s="5"/>
     </row>
-    <row r="241" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="241" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B241" s="5"/>
     </row>
-    <row r="242" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="242" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B242" s="5"/>
     </row>
-    <row r="243" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="243" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B243" s="5"/>
     </row>
-    <row r="244" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="244" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B244" s="5"/>
     </row>
-    <row r="245" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="245" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B245" s="5"/>
     </row>
-    <row r="246" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="246" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B246" s="5"/>
     </row>
-    <row r="247" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="247" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B247" s="5"/>
     </row>
-    <row r="248" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="248" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B248" s="5"/>
     </row>
-    <row r="249" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="249" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B249" s="5"/>
     </row>
-    <row r="250" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="250" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B250" s="5"/>
     </row>
-    <row r="251" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="251" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B251" s="5"/>
     </row>
-    <row r="252" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="252" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B252" s="5"/>
     </row>
-    <row r="253" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="253" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B253" s="5"/>
     </row>
-    <row r="254" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="254" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B254" s="5"/>
     </row>
-    <row r="255" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="255" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B255" s="5"/>
     </row>
-    <row r="256" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="256" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B256" s="5"/>
     </row>
-    <row r="257" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="257" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B257" s="5"/>
     </row>
-    <row r="258" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="258" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B258" s="5"/>
     </row>
-    <row r="259" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="259" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B259" s="5"/>
     </row>
-    <row r="260" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="260" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B260" s="5"/>
     </row>
-    <row r="261" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="261" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B261" s="5"/>
     </row>
-    <row r="262" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="262" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B262" s="5"/>
     </row>
-    <row r="263" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="263" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B263" s="5"/>
     </row>
-    <row r="264" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="264" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B264" s="5"/>
     </row>
-    <row r="265" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="265" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B265" s="5"/>
     </row>
-    <row r="266" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="266" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B266" s="5"/>
     </row>
-    <row r="267" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="267" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B267" s="5"/>
     </row>
-    <row r="268" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="268" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B268" s="5"/>
     </row>
-    <row r="269" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="269" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B269" s="5"/>
     </row>
-    <row r="270" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="270" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B270" s="5"/>
     </row>
-    <row r="271" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="271" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B271" s="5"/>
     </row>
-    <row r="272" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="272" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B272" s="5"/>
     </row>
-    <row r="273" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="273" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B273" s="5"/>
     </row>
-    <row r="274" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="274" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B274" s="5"/>
     </row>
-    <row r="275" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="275" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B275" s="5"/>
     </row>
-    <row r="276" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="276" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B276" s="5"/>
     </row>
-    <row r="277" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="277" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B277" s="5"/>
     </row>
-    <row r="278" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="278" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B278" s="5"/>
     </row>
-    <row r="279" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="279" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B279" s="5"/>
     </row>
-    <row r="280" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="280" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B280" s="5"/>
     </row>
-    <row r="281" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="281" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B281" s="5"/>
     </row>
-    <row r="282" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="282" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B282" s="5"/>
     </row>
-    <row r="283" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="283" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B283" s="5"/>
     </row>
-    <row r="284" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="284" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B284" s="5"/>
     </row>
-    <row r="285" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="285" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B285" s="5"/>
     </row>
-    <row r="286" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="286" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B286" s="5"/>
     </row>
-    <row r="287" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="287" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B287" s="5"/>
     </row>
-    <row r="288" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="288" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B288" s="5"/>
     </row>
-    <row r="289" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="289" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B289" s="5"/>
     </row>
-    <row r="290" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="290" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B290" s="5"/>
     </row>
-    <row r="291" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="291" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B291" s="5"/>
     </row>
-    <row r="292" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="292" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B292" s="5"/>
     </row>
-    <row r="293" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="293" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B293" s="5"/>
     </row>
-    <row r="294" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="294" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B294" s="5"/>
     </row>
-    <row r="295" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="295" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B295" s="5"/>
     </row>
-    <row r="296" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="296" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B296" s="5"/>
     </row>
-    <row r="297" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="297" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B297" s="5"/>
     </row>
-    <row r="298" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="298" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B298" s="5"/>
     </row>
-    <row r="299" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="299" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B299" s="5"/>
     </row>
-    <row r="300" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="300" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B300" s="5"/>
     </row>
-    <row r="301" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="301" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B301" s="5"/>
     </row>
-    <row r="302" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="302" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B302" s="5"/>
     </row>
-    <row r="303" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="303" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B303" s="5"/>
     </row>
-    <row r="304" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="304" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B304" s="5"/>
     </row>
-    <row r="305" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="305" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B305" s="5"/>
     </row>
-    <row r="306" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="306" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B306" s="5"/>
     </row>
-    <row r="307" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="307" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B307" s="5"/>
     </row>
-    <row r="308" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="308" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B308" s="5"/>
     </row>
-    <row r="309" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="309" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B309" s="5"/>
     </row>
-    <row r="310" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="310" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B310" s="5"/>
     </row>
-    <row r="311" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="311" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B311" s="5"/>
     </row>
-    <row r="312" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="312" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B312" s="5"/>
     </row>
-    <row r="313" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="313" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B313" s="5"/>
     </row>
-    <row r="314" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="314" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B314" s="5"/>
     </row>
-    <row r="315" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="315" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B315" s="5"/>
     </row>
-    <row r="316" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="316" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B316" s="5"/>
     </row>
-    <row r="317" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="317" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B317" s="5"/>
     </row>
-    <row r="318" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="318" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B318" s="5"/>
     </row>
-    <row r="319" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="319" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B319" s="5"/>
     </row>
-    <row r="320" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="320" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B320" s="5"/>
     </row>
-    <row r="321" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="321" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B321" s="5"/>
     </row>
-    <row r="322" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="322" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B322" s="5"/>
     </row>
-    <row r="323" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="323" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B323" s="5"/>
     </row>
-    <row r="324" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="324" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B324" s="5"/>
     </row>
-    <row r="325" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="325" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B325" s="5"/>
     </row>
-    <row r="326" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="326" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B326" s="5"/>
     </row>
-    <row r="327" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="327" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B327" s="5"/>
     </row>
-    <row r="328" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="328" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B328" s="5"/>
     </row>
-    <row r="329" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="329" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B329" s="5"/>
     </row>
-    <row r="330" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="330" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B330" s="5"/>
     </row>
-    <row r="331" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="331" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B331" s="5"/>
     </row>
-    <row r="332" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="332" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B332" s="5"/>
     </row>
-    <row r="333" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="333" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B333" s="5"/>
     </row>
-    <row r="334" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="334" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B334" s="5"/>
     </row>
-    <row r="335" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="335" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B335" s="5"/>
     </row>
-    <row r="336" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="336" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B336" s="5"/>
     </row>
-    <row r="337" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="337" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B337" s="5"/>
     </row>
-    <row r="338" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="338" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B338" s="5"/>
     </row>
-    <row r="339" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="339" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B339" s="5"/>
     </row>
-    <row r="340" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="340" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B340" s="5"/>
     </row>
-    <row r="341" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="341" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B341" s="5"/>
     </row>
-    <row r="342" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="342" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B342" s="5"/>
     </row>
-    <row r="343" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="343" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B343" s="5"/>
     </row>
-    <row r="344" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="344" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B344" s="5"/>
     </row>
-    <row r="345" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="345" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B345" s="5"/>
     </row>
-    <row r="346" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="346" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B346" s="5"/>
     </row>
-    <row r="347" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="347" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B347" s="5"/>
     </row>
-    <row r="348" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="348" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B348" s="5"/>
     </row>
-    <row r="349" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="349" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B349" s="5"/>
     </row>
-    <row r="350" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="350" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B350" s="5"/>
     </row>
-    <row r="351" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="351" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B351" s="5"/>
     </row>
-    <row r="352" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="352" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B352" s="5"/>
     </row>
-    <row r="353" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="353" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B353" s="5"/>
     </row>
-    <row r="354" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="354" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B354" s="5"/>
     </row>
-    <row r="355" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="355" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B355" s="5"/>
     </row>
-    <row r="356" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="356" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B356" s="5"/>
     </row>
-    <row r="357" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="357" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B357" s="5"/>
     </row>
-    <row r="358" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="358" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B358" s="5"/>
     </row>
-    <row r="359" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="359" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B359" s="5"/>
     </row>
-    <row r="360" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="360" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B360" s="5"/>
     </row>
-    <row r="361" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="361" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B361" s="5"/>
     </row>
-    <row r="362" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="362" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B362" s="5"/>
     </row>
-    <row r="363" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="363" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B363" s="5"/>
     </row>
-    <row r="364" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="364" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B364" s="5"/>
     </row>
-    <row r="365" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="365" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B365" s="5"/>
     </row>
-    <row r="366" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="366" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B366" s="5"/>
     </row>
-    <row r="367" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="367" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B367" s="5"/>
     </row>
-    <row r="368" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="368" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B368" s="5"/>
     </row>
-    <row r="369" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="369" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B369" s="5"/>
     </row>
-    <row r="370" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="370" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B370" s="5"/>
     </row>
-    <row r="371" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="371" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B371" s="5"/>
     </row>
-    <row r="372" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="372" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B372" s="5"/>
     </row>
-    <row r="373" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="373" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B373" s="5"/>
     </row>
-    <row r="374" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="374" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B374" s="5"/>
     </row>
-    <row r="375" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="375" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B375" s="5"/>
     </row>
-    <row r="376" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="376" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B376" s="5"/>
     </row>
-    <row r="377" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="377" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B377" s="5"/>
     </row>
-    <row r="378" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="378" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B378" s="5"/>
     </row>
-    <row r="379" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="379" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B379" s="5"/>
     </row>
-    <row r="380" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="380" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B380" s="5"/>
     </row>
-    <row r="381" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="381" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B381" s="5"/>
     </row>
-    <row r="382" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="382" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B382" s="5"/>
     </row>
-    <row r="383" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="383" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B383" s="5"/>
     </row>
-    <row r="384" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="384" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B384" s="5"/>
     </row>
-    <row r="385" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="385" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B385" s="5"/>
     </row>
-    <row r="386" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="386" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B386" s="5"/>
     </row>
-    <row r="387" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="387" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B387" s="5"/>
     </row>
-    <row r="388" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="388" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B388" s="5"/>
     </row>
-    <row r="389" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="389" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B389" s="5"/>
     </row>
-    <row r="390" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="390" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B390" s="5"/>
     </row>
-    <row r="391" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="391" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B391" s="5"/>
     </row>
-    <row r="392" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="392" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B392" s="5"/>
     </row>
-    <row r="393" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="393" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B393" s="5"/>
     </row>
-    <row r="394" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="394" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B394" s="5"/>
     </row>
-    <row r="395" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="395" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B395" s="5"/>
     </row>
-    <row r="396" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="396" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B396" s="5"/>
     </row>
-    <row r="397" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="397" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B397" s="5"/>
     </row>
-    <row r="398" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="398" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B398" s="5"/>
     </row>
-    <row r="399" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="399" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B399" s="5"/>
     </row>
-    <row r="400" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="400" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B400" s="5"/>
     </row>
-    <row r="401" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="401" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B401" s="5"/>
     </row>
-    <row r="402" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="402" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B402" s="5"/>
     </row>
-    <row r="403" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="403" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B403" s="5"/>
     </row>
-    <row r="404" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="404" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B404" s="5"/>
     </row>
-    <row r="405" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="405" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B405" s="5"/>
     </row>
-    <row r="406" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="406" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B406" s="5"/>
     </row>
-    <row r="407" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="407" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B407" s="5"/>
     </row>
-    <row r="408" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="408" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B408" s="5"/>
     </row>
-    <row r="409" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="409" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B409" s="5"/>
     </row>
-    <row r="410" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="410" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B410" s="5"/>
     </row>
-    <row r="411" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="411" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B411" s="5"/>
     </row>
-    <row r="412" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="412" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B412" s="5"/>
     </row>
-    <row r="413" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="413" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B413" s="5"/>
     </row>
-    <row r="414" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="414" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B414" s="5"/>
     </row>
-    <row r="415" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="415" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B415" s="5"/>
     </row>
-    <row r="416" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="416" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B416" s="5"/>
     </row>
-    <row r="417" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="417" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B417" s="5"/>
     </row>
-    <row r="418" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="418" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B418" s="5"/>
     </row>
-    <row r="419" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="419" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B419" s="5"/>
     </row>
-    <row r="420" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="420" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B420" s="5"/>
     </row>
-    <row r="421" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="421" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B421" s="5"/>
     </row>
-    <row r="422" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="422" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B422" s="5"/>
     </row>
-    <row r="423" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="423" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B423" s="5"/>
     </row>
-    <row r="424" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="424" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B424" s="5"/>
     </row>
-    <row r="425" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="425" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B425" s="5"/>
     </row>
-    <row r="426" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="426" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B426" s="5"/>
     </row>
-    <row r="427" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="427" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B427" s="5"/>
     </row>
-    <row r="428" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="428" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B428" s="5"/>
     </row>
-    <row r="429" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="429" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B429" s="5"/>
     </row>
-    <row r="430" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="430" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B430" s="5"/>
     </row>
-    <row r="431" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="431" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B431" s="5"/>
     </row>
-    <row r="432" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="432" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B432" s="5"/>
     </row>
-    <row r="433" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="433" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B433" s="5"/>
     </row>
-    <row r="434" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="434" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B434" s="5"/>
     </row>
-    <row r="435" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="435" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B435" s="5"/>
     </row>
-    <row r="436" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="436" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B436" s="5"/>
     </row>
-    <row r="437" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="437" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B437" s="5"/>
     </row>
-    <row r="438" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="438" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B438" s="5"/>
     </row>
-    <row r="439" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="439" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B439" s="5"/>
     </row>
-    <row r="440" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="440" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B440" s="5"/>
     </row>
-    <row r="441" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="441" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B441" s="5"/>
     </row>
-    <row r="442" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="442" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B442" s="5"/>
     </row>
-    <row r="443" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="443" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B443" s="5"/>
     </row>
-    <row r="444" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="444" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B444" s="5"/>
     </row>
-    <row r="445" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="445" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B445" s="5"/>
     </row>
-    <row r="446" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="446" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B446" s="5"/>
     </row>
-    <row r="447" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="447" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B447" s="5"/>
     </row>
-    <row r="448" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="448" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B448" s="5"/>
     </row>
-    <row r="449" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="449" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B449" s="5"/>
     </row>
-    <row r="450" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="450" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B450" s="5"/>
     </row>
-    <row r="451" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="451" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B451" s="5"/>
     </row>
-    <row r="452" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="452" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B452" s="5"/>
     </row>
-    <row r="453" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="453" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B453" s="5"/>
     </row>
-    <row r="454" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="454" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B454" s="5"/>
     </row>
-    <row r="455" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="455" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B455" s="5"/>
     </row>
-    <row r="456" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="456" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B456" s="5"/>
     </row>
-    <row r="457" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="457" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B457" s="5"/>
     </row>
-    <row r="458" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="458" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B458" s="5"/>
     </row>
-    <row r="459" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="459" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B459" s="5"/>
     </row>
-    <row r="460" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="460" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B460" s="5"/>
     </row>
-    <row r="461" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="461" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B461" s="5"/>
     </row>
-    <row r="462" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="462" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B462" s="5"/>
     </row>
-    <row r="463" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="463" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B463" s="5"/>
     </row>
-    <row r="464" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="464" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B464" s="5"/>
     </row>
-    <row r="465" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="465" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B465" s="5"/>
     </row>
-    <row r="466" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="466" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B466" s="5"/>
     </row>
-    <row r="467" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="467" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B467" s="5"/>
     </row>
-    <row r="468" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="468" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B468" s="5"/>
     </row>
-    <row r="469" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="469" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B469" s="5"/>
     </row>
-    <row r="470" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="470" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B470" s="5"/>
     </row>
-    <row r="471" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="471" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B471" s="5"/>
     </row>
-    <row r="472" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="472" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B472" s="5"/>
     </row>
-    <row r="473" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="473" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B473" s="5"/>
     </row>
-    <row r="474" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="474" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B474" s="5"/>
     </row>
-    <row r="475" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="475" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B475" s="5"/>
     </row>
-    <row r="476" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="476" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B476" s="5"/>
     </row>
-    <row r="477" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="477" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B477" s="5"/>
     </row>
-    <row r="478" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="478" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B478" s="5"/>
     </row>
-    <row r="479" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="479" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B479" s="5"/>
     </row>
-    <row r="480" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="480" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B480" s="5"/>
     </row>
-    <row r="481" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="481" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B481" s="5"/>
     </row>
-    <row r="482" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="482" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B482" s="5"/>
     </row>
-    <row r="483" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="483" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B483" s="5"/>
     </row>
-    <row r="484" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="484" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B484" s="5"/>
     </row>
-    <row r="485" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="485" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B485" s="5"/>
     </row>
-    <row r="486" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="486" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B486" s="5"/>
     </row>
-    <row r="487" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="487" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B487" s="5"/>
     </row>
-    <row r="488" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="488" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B488" s="5"/>
     </row>
-    <row r="489" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="489" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B489" s="5"/>
     </row>
-    <row r="490" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="490" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B490" s="5"/>
     </row>
-    <row r="491" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="491" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B491" s="5"/>
     </row>
-    <row r="492" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="492" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B492" s="5"/>
     </row>
-    <row r="493" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="493" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B493" s="5"/>
     </row>
-    <row r="494" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="494" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B494" s="5"/>
     </row>
-    <row r="495" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="495" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B495" s="5"/>
     </row>
-    <row r="496" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="496" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B496" s="5"/>
     </row>
-    <row r="497" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="497" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B497" s="5"/>
     </row>
-    <row r="498" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="498" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B498" s="5"/>
     </row>
-    <row r="499" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="499" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B499" s="5"/>
     </row>
-    <row r="500" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="500" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B500" s="5"/>
     </row>
-    <row r="501" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="501" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B501" s="5"/>
     </row>
-    <row r="502" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="502" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B502" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <dataValidations count="8">
+  <dataValidations count="10">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Tipo inválido" error="Selecciona Gasto o Ingreso. Si lo dejas vacío, NETO lo asume como Gasto." sqref="D10:D502">
       <formula1>"Gasto,Ingreso"</formula1>
     </dataValidation>
@@ -2117,15 +2142,21 @@
       <formula1>"Alimentación,Transporte,Vivienda,Salud,Entretenimiento,Compras,Educación,Finanzas,Trabajo_Negocio,Otros"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="F10:F502">
+      <formula1>"delivery,restaurante,supermercado,mercado,cafeteria,snacks,uber_cabify,taxi,bus_micro,metro_bus,gasolina,peaje,estacionamiento,alquiler,mantenimiento,electricidad,agua,gas,internet,cable,farmacia,medico,clinica,laboratorio,seguro_salud,optica,streaming,cine,juegos,bares_clubs,eventos,hobbies,ropa,calzado,electronico,hogar,belleza,mascotas,universidad,instituto,curso_online,utiles,idiomas,colegios,prestamo,tarjeta_credito,seguro,ahorro,inversion,comision_banco,herramientas,publicidad,oficina,logistica,contador,regalo,donacion,multa,viaje,sin_categoria"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="F3:F502">
+      <formula1>"delivery,restaurante,supermercado,mercado,cafeteria,snacks,uber_cabify,taxi,bus_micro,metro_bus,gasolina,peaje,estacionamiento,alquiler,mantenimiento,electricidad,agua,gas,internet,cable,farmacia,medico,clinica,laboratorio,seguro_salud,optica,streaming,cine,juegos,bares_clubs,eventos,hobbies,ropa,calzado,electronico,hogar,belleza,mascotas,universidad,instituto,curso_online,utiles,idiomas,colegios,prestamo,tarjeta_credito,seguro,ahorro,inversion,comision_banco,herramientas,publicidad,oficina,logistica,contador,regalo,donacion,multa,viaje,sin_categoria"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="G10:G502">
       <formula1>"Yape,Plin,Débito,Crédito,Efectivo,Transferencia,Otro"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="F3:F502">
+    <dataValidation type="list" allowBlank="1" sqref="G3:G502">
       <formula1>"Yape,Plin,Débito,Crédito,Efectivo,Transferencia,Otro"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="G10:G502">
+    <dataValidation type="list" allowBlank="1" sqref="H10:H502">
       <formula1>"BCP,Interbank,BBVA,Scotiabank,Yape,Plin,Otro"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="G3:G502">
+    <dataValidation type="list" allowBlank="1" sqref="H3:H502">
       <formula1>"BCP,Interbank,BBVA,Scotiabank,Yape,Plin,Otro"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>